<commit_message>
Close #112 add hint to dataset form and excel sample
</commit_message>
<xml_diff>
--- a/public/dataset_sample.xlsx
+++ b/public/dataset_sample.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="27011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10215"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/www/csc-webportal/public/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sokly/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90ADF837-BF00-D54C-A9DF-A567AC12AE9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="14380" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="25600" windowHeight="14380" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Koh Kong" sheetId="1" r:id="rId1"/>
     <sheet name="Kratie" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0" concurrentCalc="0"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
@@ -28,12 +29,13 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Microsoft Office User</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -41,12 +43,20 @@
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>Must follow NCDD location id (commune_id, district_id) in Englishhttp://db.ncdd.gov.kh/gazetteer/view/index.castle
-	-Sokly Heng</t>
+          <t xml:space="preserve">Must follow NCDD location id (commune_id, district_id) in Englishhttp://db.ncdd.gov.kh/gazetteer/view/index.castle
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">	-Sokly Heng</t>
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -54,12 +64,199 @@
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
           </rPr>
-          <t>if school code present, then we will find for this code to update or create new record following this school code.
-In case school code is not present, then the system will used the generate a new school code for this record following the format.
-commune_code_auto-increment_id_from_previous_commune_code
-e.g: commune code is 090101 -&gt; and this school is the first in this commune -&gt;
-school code is 090101_1
-	-Sokly Heng</t>
+          <t xml:space="preserve">if school code present, then we will find for this code to update or create new record following this school code.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">In case school code is not present, then the system will used the generate a new school code for this record following the format.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">commune_code_auto-increment_id_from_previous_commune_code
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">e.g: commune code is 090101 -&gt; and this school is the first in this commune -&gt;
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">school code is 090101_1
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">	-Sokly Heng</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="1" shapeId="0" xr:uid="{A76D5855-E76F-374C-BD82-20EAAC4560F5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Microsoft Office User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">បញ្ចូលតែឈ្មោះជាភាសាអង់គ្លេស (កុំដាក់ឈ្មោះ </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t>Category)</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t>។ ឧ៖ “</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t>Srae Thmey Primary School” → “Srae Thmey”</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="1" shapeId="0" xr:uid="{23C920BA-928A-8340-9C43-FE5DF6176083}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Microsoft Office User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">បញ្ចូលតែឈ្មោះជាភាសាខ្មែរ (កុំដាក់ឈ្មោះ </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t>Category)</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t xml:space="preserve">។ ឧ៖ “បឋមសិក្សាស្រែថ្មី” </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t>→ “</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+          </rPr>
+          <t>ស្រែថ្មី”</t>
         </r>
       </text>
     </comment>
@@ -68,12 +265,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
       <text>
         <r>
           <rPr>
@@ -86,7 +283,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
       <text>
         <r>
           <rPr>
@@ -185,8 +382,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="11" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -240,6 +437,19 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -269,7 +479,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="16">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -285,16 +495,16 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -306,6 +516,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -508,12 +721,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr enableFormatConditionsCalculation="0">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:W4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18.1640625" style="9" customWidth="1"/>
     <col min="2" max="2" width="17" style="9" customWidth="1"/>
@@ -521,7 +734,7 @@
     <col min="4" max="4" width="19.83203125" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:23" ht="15.75" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>23</v>
       </c>
@@ -554,7 +767,7 @@
       <c r="V1" s="1"/>
       <c r="W1" s="1"/>
     </row>
-    <row r="2" spans="1:23" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:23" ht="16">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
@@ -569,7 +782,7 @@
       </c>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:23" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:23" ht="16">
       <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
@@ -583,7 +796,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:23" ht="16">
       <c r="A4" s="6" t="s">
         <v>0</v>
       </c>
@@ -604,12 +817,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr enableFormatConditionsCalculation="0">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:W5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18.1640625" style="9" customWidth="1"/>
     <col min="2" max="2" width="14.5" style="9" customWidth="1"/>
@@ -617,7 +830,7 @@
     <col min="4" max="4" width="20.5" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:23" ht="15.75" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>23</v>
       </c>
@@ -650,7 +863,7 @@
       <c r="V1" s="3"/>
       <c r="W1" s="3"/>
     </row>
-    <row r="2" spans="1:23" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:23" ht="26">
       <c r="A2" s="11" t="s">
         <v>10</v>
       </c>
@@ -664,7 +877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:23" ht="26">
       <c r="A3" s="11" t="s">
         <v>10</v>
       </c>
@@ -678,7 +891,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:23" ht="26">
       <c r="A4" s="11" t="s">
         <v>10</v>
       </c>
@@ -692,7 +905,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:23" ht="15.75" customHeight="1">
       <c r="A5" s="14"/>
       <c r="B5" s="14"/>
       <c r="C5" s="15"/>

</xml_diff>